<commit_message>
docs(excel): show every excel chart type in the gallery
The Excel gallery lists every chart type and what it is read as, and
gains stock, histogram, box and whisker, radar, waterfall and treemap
examples. sales.xlsx gains four sheets, which excel_example.py writes,
swapping placeholder parts for the chartEx parts XlsxWriter cannot
write; it still regenerates the file byte for byte.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkpSSRfCkBz7sveSn4KpNa
</commit_message>
<xml_diff>
--- a/docs/sales.xlsx
+++ b/docs/sales.xlsx
@@ -8,13 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
+    <sheet name="Scores" sheetId="3" r:id="rId3"/>
+    <sheet name="Budget" sheetId="4" r:id="rId4"/>
+    <sheet name="Products" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="38">
   <si>
     <t>Quarter</t>
   </si>
@@ -38,14 +42,105 @@
   </si>
   <si>
     <t>Q4</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Class A</t>
+  </si>
+  <si>
+    <t>Class B</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Amount ($k)</t>
+  </si>
+  <si>
+    <t>Opening balance</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>Tax</t>
+  </si>
+  <si>
+    <t>Closing balance</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Fruit</t>
+  </si>
+  <si>
+    <t>Apples</t>
+  </si>
+  <si>
+    <t>Pears</t>
+  </si>
+  <si>
+    <t>Plums</t>
+  </si>
+  <si>
+    <t>Vegetables</t>
+  </si>
+  <si>
+    <t>Carrots</t>
+  </si>
+  <si>
+    <t>Kale</t>
+  </si>
+  <si>
+    <t>Bakery</t>
+  </si>
+  <si>
+    <t>Bread</t>
+  </si>
+  <si>
+    <t>Cakes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0%"/>
+    <numFmt numFmtId="165" formatCode="mmm d"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -84,10 +179,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -296,6 +392,142 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Budget!$A$2:$A$8</cx:f>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Opening balance</cx:pt>
+          <cx:pt idx="1">Sales</cx:pt>
+          <cx:pt idx="2">Services</cx:pt>
+          <cx:pt idx="3">Salaries</cx:pt>
+          <cx:pt idx="4">Rent</cx:pt>
+          <cx:pt idx="5">Tax</cx:pt>
+          <cx:pt idx="6">Closing balance</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>Budget!$B$2:$B$8</cx:f>
+        <cx:lvl ptCount="7" formatCode="General">
+          <cx:pt idx="0">500</cx:pt>
+          <cx:pt idx="1">320</cx:pt>
+          <cx:pt idx="2">140</cx:pt>
+          <cx:pt idx="3">-380</cx:pt>
+          <cx:pt idx="4">-90</cx:pt>
+          <cx:pt idx="5">-60</cx:pt>
+          <cx:pt idx="6">430</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Cash flow</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="waterfall">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Amount ($k)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:subtotals>
+              <cx:idx val="0"/>
+              <cx:idx val="6"/>
+            </cx:subtotals>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Products!$A$2:$B$8</cx:f>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Apples</cx:pt>
+          <cx:pt idx="1">Pears</cx:pt>
+          <cx:pt idx="2">Plums</cx:pt>
+          <cx:pt idx="3">Carrots</cx:pt>
+          <cx:pt idx="4">Kale</cx:pt>
+          <cx:pt idx="5">Bread</cx:pt>
+          <cx:pt idx="6">Cakes</cx:pt>
+        </cx:lvl>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Fruit</cx:pt>
+          <cx:pt idx="1">Fruit</cx:pt>
+          <cx:pt idx="2">Fruit</cx:pt>
+          <cx:pt idx="3">Vegetables</cx:pt>
+          <cx:pt idx="4">Vegetables</cx:pt>
+          <cx:pt idx="5">Bakery</cx:pt>
+          <cx:pt idx="6">Bakery</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="size">
+        <cx:f>Products!$C$2:$C$8</cx:f>
+        <cx:lvl ptCount="7" formatCode="General">
+          <cx:pt idx="0">120</cx:pt>
+          <cx:pt idx="1">60</cx:pt>
+          <cx:pt idx="2">30</cx:pt>
+          <cx:pt idx="3">80</cx:pt>
+          <cx:pt idx="4">40</cx:pt>
+          <cx:pt idx="5">90</cx:pt>
+          <cx:pt idx="6">50</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Sales by product</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="treemap">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Sales</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr/>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -994,6 +1226,714 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue around the year</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sales!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sales!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>175</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sales!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>South</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sales!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$C$2:$C$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>160</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="50060001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50060002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="cross"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Share price, first week of January</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:stockChart>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Open</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>41.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>41.4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>43.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>High</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44.8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45.6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="dot"/>
+            <c:size val="3"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$D$2:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>40.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>41.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>41.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>43.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>43.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Close</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$E$2:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>42.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>41.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>43.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:hiLowLines/>
+        <c:upDownBars>
+          <c:gapWidth val="150"/>
+          <c:upBars/>
+          <c:downBars/>
+        </c:upDownBars>
+        <c:axId val="50070001"/>
+        <c:axId val="50070002"/>
+      </c:stockChart>
+      <c:dateAx>
+        <c:axId val="50070001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm d" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50070002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="50070002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50070001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>Scores!$B$2:$B$28</cx:f>
+        <cx:lvl ptCount="27" formatCode="General">
+          <cx:pt idx="0">52</cx:pt>
+          <cx:pt idx="1">58</cx:pt>
+          <cx:pt idx="2">61</cx:pt>
+          <cx:pt idx="3">64</cx:pt>
+          <cx:pt idx="4">66</cx:pt>
+          <cx:pt idx="5">68</cx:pt>
+          <cx:pt idx="6">70</cx:pt>
+          <cx:pt idx="7">71</cx:pt>
+          <cx:pt idx="8">73</cx:pt>
+          <cx:pt idx="9">75</cx:pt>
+          <cx:pt idx="10">77</cx:pt>
+          <cx:pt idx="11">80</cx:pt>
+          <cx:pt idx="12">84</cx:pt>
+          <cx:pt idx="13">97</cx:pt>
+          <cx:pt idx="14">45</cx:pt>
+          <cx:pt idx="15">55</cx:pt>
+          <cx:pt idx="16">59</cx:pt>
+          <cx:pt idx="17">62</cx:pt>
+          <cx:pt idx="18">63</cx:pt>
+          <cx:pt idx="19">67</cx:pt>
+          <cx:pt idx="20">69</cx:pt>
+          <cx:pt idx="21">72</cx:pt>
+          <cx:pt idx="22">74</cx:pt>
+          <cx:pt idx="23">78</cx:pt>
+          <cx:pt idx="24">79</cx:pt>
+          <cx:pt idx="25">83</cx:pt>
+          <cx:pt idx="26">88</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Scores, both classes</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Score</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binSize val="10"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Scores!$A$2:$A$28</cx:f>
+        <cx:lvl ptCount="27">
+          <cx:pt idx="0">Class A</cx:pt>
+          <cx:pt idx="1">Class A</cx:pt>
+          <cx:pt idx="2">Class A</cx:pt>
+          <cx:pt idx="3">Class A</cx:pt>
+          <cx:pt idx="4">Class A</cx:pt>
+          <cx:pt idx="5">Class A</cx:pt>
+          <cx:pt idx="6">Class A</cx:pt>
+          <cx:pt idx="7">Class A</cx:pt>
+          <cx:pt idx="8">Class A</cx:pt>
+          <cx:pt idx="9">Class A</cx:pt>
+          <cx:pt idx="10">Class A</cx:pt>
+          <cx:pt idx="11">Class A</cx:pt>
+          <cx:pt idx="12">Class A</cx:pt>
+          <cx:pt idx="13">Class A</cx:pt>
+          <cx:pt idx="14">Class B</cx:pt>
+          <cx:pt idx="15">Class B</cx:pt>
+          <cx:pt idx="16">Class B</cx:pt>
+          <cx:pt idx="17">Class B</cx:pt>
+          <cx:pt idx="18">Class B</cx:pt>
+          <cx:pt idx="19">Class B</cx:pt>
+          <cx:pt idx="20">Class B</cx:pt>
+          <cx:pt idx="21">Class B</cx:pt>
+          <cx:pt idx="22">Class B</cx:pt>
+          <cx:pt idx="23">Class B</cx:pt>
+          <cx:pt idx="24">Class B</cx:pt>
+          <cx:pt idx="25">Class B</cx:pt>
+          <cx:pt idx="26">Class B</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>Scores!$B$2:$B$28</cx:f>
+        <cx:lvl ptCount="27" formatCode="General">
+          <cx:pt idx="0">52</cx:pt>
+          <cx:pt idx="1">58</cx:pt>
+          <cx:pt idx="2">61</cx:pt>
+          <cx:pt idx="3">64</cx:pt>
+          <cx:pt idx="4">66</cx:pt>
+          <cx:pt idx="5">68</cx:pt>
+          <cx:pt idx="6">70</cx:pt>
+          <cx:pt idx="7">71</cx:pt>
+          <cx:pt idx="8">73</cx:pt>
+          <cx:pt idx="9">75</cx:pt>
+          <cx:pt idx="10">77</cx:pt>
+          <cx:pt idx="11">80</cx:pt>
+          <cx:pt idx="12">84</cx:pt>
+          <cx:pt idx="13">97</cx:pt>
+          <cx:pt idx="14">45</cx:pt>
+          <cx:pt idx="15">55</cx:pt>
+          <cx:pt idx="16">59</cx:pt>
+          <cx:pt idx="17">62</cx:pt>
+          <cx:pt idx="18">63</cx:pt>
+          <cx:pt idx="19">67</cx:pt>
+          <cx:pt idx="20">69</cx:pt>
+          <cx:pt idx="21">72</cx:pt>
+          <cx:pt idx="22">74</cx:pt>
+          <cx:pt idx="23">78</cx:pt>
+          <cx:pt idx="24">79</cx:pt>
+          <cx:pt idx="25">83</cx:pt>
+          <cx:pt idx="26">88</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Scores by class</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Score</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1143,6 +2083,206 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1513,4 +2653,526 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="3">
+        <v>46027</v>
+      </c>
+      <c r="B2">
+        <v>41.2</v>
+      </c>
+      <c r="C2">
+        <v>43</v>
+      </c>
+      <c r="D2">
+        <v>40.6</v>
+      </c>
+      <c r="E2">
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="3">
+        <v>46028</v>
+      </c>
+      <c r="B3">
+        <v>42.5</v>
+      </c>
+      <c r="C3">
+        <v>42.9</v>
+      </c>
+      <c r="D3">
+        <v>41.1</v>
+      </c>
+      <c r="E3">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="3">
+        <v>46029</v>
+      </c>
+      <c r="B4">
+        <v>41.4</v>
+      </c>
+      <c r="C4">
+        <v>44.2</v>
+      </c>
+      <c r="D4">
+        <v>41.3</v>
+      </c>
+      <c r="E4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3">
+        <v>46030</v>
+      </c>
+      <c r="B5">
+        <v>44</v>
+      </c>
+      <c r="C5">
+        <v>44.8</v>
+      </c>
+      <c r="D5">
+        <v>43.1</v>
+      </c>
+      <c r="E5">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="3">
+        <v>46031</v>
+      </c>
+      <c r="B6">
+        <v>43.5</v>
+      </c>
+      <c r="C6">
+        <v>45.6</v>
+      </c>
+      <c r="D6">
+        <v>43.4</v>
+      </c>
+      <c r="E6">
+        <v>45.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>-380</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7">
+        <v>-60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8">
+        <v>430</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(excel): read every chart type excel draws (#859)
read_excel_charts now reads stacked line, radar, bubble, stock, surface
and pie-of-pie charts, and the Excel 2016 types kept in chartEx parts:
histogram, Pareto, box and whisker, waterfall, funnel, treemap, sunburst
and map. Where matplotlib has a call for a chart it is drawn through the
patched Axes call; where it has none, the marks are drawn from plain
artists and an ExcelLayer built from the chart's values is registered
through FigureManager.add_plot. Histogram bins and box quartiles are
worked out as Excel works them out; a map is read as its region list. A
stock chart's volume is also read as a bar layer of its own. The Excel
gallery shows the new types.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkpSSRfCkBz7sveSn4KpNa
</commit_message>
<xml_diff>
--- a/docs/sales.xlsx
+++ b/docs/sales.xlsx
@@ -8,13 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
+    <sheet name="Scores" sheetId="3" r:id="rId3"/>
+    <sheet name="Budget" sheetId="4" r:id="rId4"/>
+    <sheet name="Products" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="38">
   <si>
     <t>Quarter</t>
   </si>
@@ -38,14 +42,105 @@
   </si>
   <si>
     <t>Q4</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Class A</t>
+  </si>
+  <si>
+    <t>Class B</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Amount ($k)</t>
+  </si>
+  <si>
+    <t>Opening balance</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>Tax</t>
+  </si>
+  <si>
+    <t>Closing balance</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Fruit</t>
+  </si>
+  <si>
+    <t>Apples</t>
+  </si>
+  <si>
+    <t>Pears</t>
+  </si>
+  <si>
+    <t>Plums</t>
+  </si>
+  <si>
+    <t>Vegetables</t>
+  </si>
+  <si>
+    <t>Carrots</t>
+  </si>
+  <si>
+    <t>Kale</t>
+  </si>
+  <si>
+    <t>Bakery</t>
+  </si>
+  <si>
+    <t>Bread</t>
+  </si>
+  <si>
+    <t>Cakes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0%"/>
+    <numFmt numFmtId="165" formatCode="mmm d"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -84,10 +179,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -296,6 +392,142 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Budget!$A$2:$A$8</cx:f>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Opening balance</cx:pt>
+          <cx:pt idx="1">Sales</cx:pt>
+          <cx:pt idx="2">Services</cx:pt>
+          <cx:pt idx="3">Salaries</cx:pt>
+          <cx:pt idx="4">Rent</cx:pt>
+          <cx:pt idx="5">Tax</cx:pt>
+          <cx:pt idx="6">Closing balance</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>Budget!$B$2:$B$8</cx:f>
+        <cx:lvl ptCount="7" formatCode="General">
+          <cx:pt idx="0">500</cx:pt>
+          <cx:pt idx="1">320</cx:pt>
+          <cx:pt idx="2">140</cx:pt>
+          <cx:pt idx="3">-380</cx:pt>
+          <cx:pt idx="4">-90</cx:pt>
+          <cx:pt idx="5">-60</cx:pt>
+          <cx:pt idx="6">430</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Cash flow</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="waterfall">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Amount ($k)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:subtotals>
+              <cx:idx val="0"/>
+              <cx:idx val="6"/>
+            </cx:subtotals>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Products!$A$2:$B$8</cx:f>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Apples</cx:pt>
+          <cx:pt idx="1">Pears</cx:pt>
+          <cx:pt idx="2">Plums</cx:pt>
+          <cx:pt idx="3">Carrots</cx:pt>
+          <cx:pt idx="4">Kale</cx:pt>
+          <cx:pt idx="5">Bread</cx:pt>
+          <cx:pt idx="6">Cakes</cx:pt>
+        </cx:lvl>
+        <cx:lvl ptCount="7">
+          <cx:pt idx="0">Fruit</cx:pt>
+          <cx:pt idx="1">Fruit</cx:pt>
+          <cx:pt idx="2">Fruit</cx:pt>
+          <cx:pt idx="3">Vegetables</cx:pt>
+          <cx:pt idx="4">Vegetables</cx:pt>
+          <cx:pt idx="5">Bakery</cx:pt>
+          <cx:pt idx="6">Bakery</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="size">
+        <cx:f>Products!$C$2:$C$8</cx:f>
+        <cx:lvl ptCount="7" formatCode="General">
+          <cx:pt idx="0">120</cx:pt>
+          <cx:pt idx="1">60</cx:pt>
+          <cx:pt idx="2">30</cx:pt>
+          <cx:pt idx="3">80</cx:pt>
+          <cx:pt idx="4">40</cx:pt>
+          <cx:pt idx="5">90</cx:pt>
+          <cx:pt idx="6">50</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Sales by product</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="treemap">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Sales</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr/>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -994,6 +1226,714 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue around the year</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sales!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sales!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>175</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sales!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>South</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sales!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sales!$C$2:$C$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>160</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="50060001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50060002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="cross"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Share price, first week of January</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:stockChart>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Open</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>41.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>41.4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>43.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>High</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44.8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45.6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="dot"/>
+            <c:size val="3"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$D$2:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>40.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>41.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>41.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>43.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>43.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prices!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Close</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:numRef>
+              <c:f>Prices!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46028</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46029</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46030</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46031</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Prices!$E$2:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>42.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>41.4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>43.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:hiLowLines/>
+        <c:upDownBars>
+          <c:gapWidth val="150"/>
+          <c:upBars/>
+          <c:downBars/>
+        </c:upDownBars>
+        <c:axId val="50070001"/>
+        <c:axId val="50070002"/>
+      </c:stockChart>
+      <c:dateAx>
+        <c:axId val="50070001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm d" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50070002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="50070002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50070001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>Scores!$B$2:$B$28</cx:f>
+        <cx:lvl ptCount="27" formatCode="General">
+          <cx:pt idx="0">52</cx:pt>
+          <cx:pt idx="1">58</cx:pt>
+          <cx:pt idx="2">61</cx:pt>
+          <cx:pt idx="3">64</cx:pt>
+          <cx:pt idx="4">66</cx:pt>
+          <cx:pt idx="5">68</cx:pt>
+          <cx:pt idx="6">70</cx:pt>
+          <cx:pt idx="7">71</cx:pt>
+          <cx:pt idx="8">73</cx:pt>
+          <cx:pt idx="9">75</cx:pt>
+          <cx:pt idx="10">77</cx:pt>
+          <cx:pt idx="11">80</cx:pt>
+          <cx:pt idx="12">84</cx:pt>
+          <cx:pt idx="13">97</cx:pt>
+          <cx:pt idx="14">45</cx:pt>
+          <cx:pt idx="15">55</cx:pt>
+          <cx:pt idx="16">59</cx:pt>
+          <cx:pt idx="17">62</cx:pt>
+          <cx:pt idx="18">63</cx:pt>
+          <cx:pt idx="19">67</cx:pt>
+          <cx:pt idx="20">69</cx:pt>
+          <cx:pt idx="21">72</cx:pt>
+          <cx:pt idx="22">74</cx:pt>
+          <cx:pt idx="23">78</cx:pt>
+          <cx:pt idx="24">79</cx:pt>
+          <cx:pt idx="25">83</cx:pt>
+          <cx:pt idx="26">88</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Scores, both classes</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Score</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binSize val="10"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>Scores!$A$2:$A$28</cx:f>
+        <cx:lvl ptCount="27">
+          <cx:pt idx="0">Class A</cx:pt>
+          <cx:pt idx="1">Class A</cx:pt>
+          <cx:pt idx="2">Class A</cx:pt>
+          <cx:pt idx="3">Class A</cx:pt>
+          <cx:pt idx="4">Class A</cx:pt>
+          <cx:pt idx="5">Class A</cx:pt>
+          <cx:pt idx="6">Class A</cx:pt>
+          <cx:pt idx="7">Class A</cx:pt>
+          <cx:pt idx="8">Class A</cx:pt>
+          <cx:pt idx="9">Class A</cx:pt>
+          <cx:pt idx="10">Class A</cx:pt>
+          <cx:pt idx="11">Class A</cx:pt>
+          <cx:pt idx="12">Class A</cx:pt>
+          <cx:pt idx="13">Class A</cx:pt>
+          <cx:pt idx="14">Class B</cx:pt>
+          <cx:pt idx="15">Class B</cx:pt>
+          <cx:pt idx="16">Class B</cx:pt>
+          <cx:pt idx="17">Class B</cx:pt>
+          <cx:pt idx="18">Class B</cx:pt>
+          <cx:pt idx="19">Class B</cx:pt>
+          <cx:pt idx="20">Class B</cx:pt>
+          <cx:pt idx="21">Class B</cx:pt>
+          <cx:pt idx="22">Class B</cx:pt>
+          <cx:pt idx="23">Class B</cx:pt>
+          <cx:pt idx="24">Class B</cx:pt>
+          <cx:pt idx="25">Class B</cx:pt>
+          <cx:pt idx="26">Class B</cx:pt>
+        </cx:lvl>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>Scores!$B$2:$B$28</cx:f>
+        <cx:lvl ptCount="27" formatCode="General">
+          <cx:pt idx="0">52</cx:pt>
+          <cx:pt idx="1">58</cx:pt>
+          <cx:pt idx="2">61</cx:pt>
+          <cx:pt idx="3">64</cx:pt>
+          <cx:pt idx="4">66</cx:pt>
+          <cx:pt idx="5">68</cx:pt>
+          <cx:pt idx="6">70</cx:pt>
+          <cx:pt idx="7">71</cx:pt>
+          <cx:pt idx="8">73</cx:pt>
+          <cx:pt idx="9">75</cx:pt>
+          <cx:pt idx="10">77</cx:pt>
+          <cx:pt idx="11">80</cx:pt>
+          <cx:pt idx="12">84</cx:pt>
+          <cx:pt idx="13">97</cx:pt>
+          <cx:pt idx="14">45</cx:pt>
+          <cx:pt idx="15">55</cx:pt>
+          <cx:pt idx="16">59</cx:pt>
+          <cx:pt idx="17">62</cx:pt>
+          <cx:pt idx="18">63</cx:pt>
+          <cx:pt idx="19">67</cx:pt>
+          <cx:pt idx="20">69</cx:pt>
+          <cx:pt idx="21">72</cx:pt>
+          <cx:pt idx="22">74</cx:pt>
+          <cx:pt idx="23">78</cx:pt>
+          <cx:pt idx="24">79</cx:pt>
+          <cx:pt idx="25">83</cx:pt>
+          <cx:pt idx="26">88</cx:pt>
+        </cx:lvl>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title>
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Scores by class</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Score</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1143,6 +2083,206 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1513,4 +2653,526 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="3">
+        <v>46027</v>
+      </c>
+      <c r="B2">
+        <v>41.2</v>
+      </c>
+      <c r="C2">
+        <v>43</v>
+      </c>
+      <c r="D2">
+        <v>40.6</v>
+      </c>
+      <c r="E2">
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="3">
+        <v>46028</v>
+      </c>
+      <c r="B3">
+        <v>42.5</v>
+      </c>
+      <c r="C3">
+        <v>42.9</v>
+      </c>
+      <c r="D3">
+        <v>41.1</v>
+      </c>
+      <c r="E3">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="3">
+        <v>46029</v>
+      </c>
+      <c r="B4">
+        <v>41.4</v>
+      </c>
+      <c r="C4">
+        <v>44.2</v>
+      </c>
+      <c r="D4">
+        <v>41.3</v>
+      </c>
+      <c r="E4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3">
+        <v>46030</v>
+      </c>
+      <c r="B5">
+        <v>44</v>
+      </c>
+      <c r="C5">
+        <v>44.8</v>
+      </c>
+      <c r="D5">
+        <v>43.1</v>
+      </c>
+      <c r="E5">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="3">
+        <v>46031</v>
+      </c>
+      <c r="B6">
+        <v>43.5</v>
+      </c>
+      <c r="C6">
+        <v>45.6</v>
+      </c>
+      <c r="D6">
+        <v>43.4</v>
+      </c>
+      <c r="E6">
+        <v>45.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>-380</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7">
+        <v>-60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8">
+        <v>430</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>